<commit_message>
Script_9: order cell types epithelial, endothelial, mesenchymal, immune
- Marker-score analysis: one cell_order in step 2 sets the order of all
  tables and the heatmap; step 1 query list uses the same order
- Region-protein analysis: endothelial compartment now precedes stromal
- Outputs regenerated; scores, statistics and FDRs are unchanged
</commit_message>
<xml_diff>
--- a/Script_9_region_cell_type_enrichment_with_scRNAseq/region protein marker in scRNAseq cell type/cell_type_signature_scores.xlsx
+++ b/Script_9_region_cell_type_enrichment_with_scRNAseq/region protein marker in scRNAseq cell type/cell_type_signature_scores.xlsx
@@ -495,48 +495,48 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Fibroblast</t>
+          <t>Capillary endothelial</t>
         </is>
       </c>
       <c r="B6">
-        <v>0.08847442751918973</v>
+        <v>-0.06598697161583275</v>
       </c>
       <c r="C6">
-        <v>-0.009090894665565464</v>
+        <v>0.1334756586371784</v>
       </c>
       <c r="D6">
-        <v>0.4394618552265902</v>
+        <v>0.2427317719460537</v>
       </c>
       <c r="E6">
-        <v>0.0602367937296894</v>
+        <v>-0.07297379478163291</v>
       </c>
       <c r="F6">
-        <v>0.1325639852261914</v>
+        <v>1.090075713263977</v>
       </c>
       <c r="G6">
-        <v>0.2860849992140306</v>
+        <v>-0.009555060828546737</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Smooth muscle</t>
+          <t>Vascular endothelial</t>
         </is>
       </c>
       <c r="B7">
-        <v>0.1985751255752783</v>
+        <v>-0.1175452845423405</v>
       </c>
       <c r="C7">
-        <v>-0.09452915772079987</v>
+        <v>-0.04119142136089762</v>
       </c>
       <c r="D7">
-        <v>0.2546304044146597</v>
+        <v>-0.05785662564583817</v>
       </c>
       <c r="E7">
-        <v>0.1011550234308974</v>
+        <v>-0.0747906881219244</v>
       </c>
       <c r="F7">
-        <v>0.02701309016729691</v>
+        <v>0.4486705216004974</v>
       </c>
       <c r="G7">
         <v>-0.009555060828546737</v>
@@ -545,23 +545,23 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Mesothelial</t>
+          <t>VCAM1+ endothelial</t>
         </is>
       </c>
       <c r="B8">
-        <v>0.178421533899693</v>
+        <v>-0.01054659966475042</v>
       </c>
       <c r="C8">
-        <v>0.03062944802439096</v>
+        <v>-0.02287353670061724</v>
       </c>
       <c r="D8">
-        <v>0.2148802125088622</v>
+        <v>0.2747744423773382</v>
       </c>
       <c r="E8">
-        <v>0.1069673843119863</v>
+        <v>0.005933938258926822</v>
       </c>
       <c r="F8">
-        <v>0.2148013491225918</v>
+        <v>0.2182824608660536</v>
       </c>
       <c r="G8">
         <v>-0.009555060828546737</v>
@@ -570,48 +570,48 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Capillary endothelial</t>
+          <t>Fibroblast</t>
         </is>
       </c>
       <c r="B9">
-        <v>-0.06598697161583275</v>
+        <v>0.08847442751918973</v>
       </c>
       <c r="C9">
-        <v>0.1334756586371784</v>
+        <v>-0.009090894665565464</v>
       </c>
       <c r="D9">
-        <v>0.2427317719460537</v>
+        <v>0.4394618552265902</v>
       </c>
       <c r="E9">
-        <v>-0.07297379478163291</v>
+        <v>0.0602367937296894</v>
       </c>
       <c r="F9">
-        <v>1.090075713263977</v>
+        <v>0.1325639852261914</v>
       </c>
       <c r="G9">
-        <v>-0.009555060828546737</v>
+        <v>0.2860849992140306</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Vascular endothelial</t>
+          <t>Smooth muscle</t>
         </is>
       </c>
       <c r="B10">
-        <v>-0.1175452845423405</v>
+        <v>0.1985751255752783</v>
       </c>
       <c r="C10">
-        <v>-0.04119142136089762</v>
+        <v>-0.09452915772079987</v>
       </c>
       <c r="D10">
-        <v>-0.05785662564583817</v>
+        <v>0.2546304044146597</v>
       </c>
       <c r="E10">
-        <v>-0.0747906881219244</v>
+        <v>0.1011550234308974</v>
       </c>
       <c r="F10">
-        <v>0.4486705216004974</v>
+        <v>0.02701309016729691</v>
       </c>
       <c r="G10">
         <v>-0.009555060828546737</v>
@@ -620,23 +620,23 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>VCAM1+ endothelial</t>
+          <t>Mesothelial</t>
         </is>
       </c>
       <c r="B11">
-        <v>-0.01054659966475042</v>
+        <v>0.178421533899693</v>
       </c>
       <c r="C11">
-        <v>-0.02287353670061724</v>
+        <v>0.03062944802439096</v>
       </c>
       <c r="D11">
-        <v>0.2747744423773382</v>
+        <v>0.2148802125088622</v>
       </c>
       <c r="E11">
-        <v>0.005933938258926822</v>
+        <v>0.1069673843119863</v>
       </c>
       <c r="F11">
-        <v>0.2182824608660536</v>
+        <v>0.2148013491225918</v>
       </c>
       <c r="G11">
         <v>-0.009555060828546737</v>
@@ -992,51 +992,51 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Stromal</t>
+          <t>Endothelial</t>
         </is>
       </c>
       <c r="B3">
-        <v>0.1398101640778449</v>
+        <v>-0.0920141923782359</v>
       </c>
       <c r="C3">
-        <v>-0.03129829223538694</v>
+        <v>-0.01581411231540799</v>
       </c>
       <c r="D3">
-        <v>0.3414374726512251</v>
+        <v>0.03928511861325036</v>
       </c>
       <c r="E3">
-        <v>0.08145665229889611</v>
+        <v>-0.06022581161422102</v>
       </c>
       <c r="F3">
-        <v>0.1104676344875204</v>
+        <v>0.4890038447898664</v>
       </c>
       <c r="G3">
-        <v>0.1395283882527521</v>
+        <v>-0.009555060828546737</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Endothelial</t>
+          <t>Stromal</t>
         </is>
       </c>
       <c r="B4">
-        <v>-0.0920141923782359</v>
+        <v>0.1398101640778449</v>
       </c>
       <c r="C4">
-        <v>-0.01581411231540799</v>
+        <v>-0.03129829223538694</v>
       </c>
       <c r="D4">
-        <v>0.03928511861325036</v>
+        <v>0.3414374726512251</v>
       </c>
       <c r="E4">
-        <v>-0.06022581161422102</v>
+        <v>0.08145665229889611</v>
       </c>
       <c r="F4">
-        <v>0.4890038447898664</v>
+        <v>0.1104676344875204</v>
       </c>
       <c r="G4">
-        <v>-0.009555060828546737</v>
+        <v>0.1395283882527521</v>
       </c>
     </row>
     <row r="5">

</xml_diff>